<commit_message>
Updating PMP test plan
</commit_message>
<xml_diff>
--- a/testplans/RV64PMP.xlsx
+++ b/testplans/RV64PMP.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="177">
   <si>
     <t>Sr No
 (link to coverage)</t>
@@ -39,7 +39,7 @@
     <t>Comments</t>
   </si>
   <si>
-    <t>cfg.3</t>
+    <t>cfg.1</t>
   </si>
   <si>
     <t>L</t>
@@ -61,14 +61,14 @@
     <t>Uncovered</t>
   </si>
   <si>
-    <t>cfg.4</t>
+    <t>cfg.2</t>
   </si>
   <si>
     <t xml:space="preserve">Perform all of the R/W/X tests below with L=1 and in M mode.
 </t>
   </si>
   <si>
-    <t>cfg.5</t>
+    <t>cfg.3</t>
   </si>
   <si>
     <t>X</t>
@@ -78,20 +78,20 @@
 </t>
   </si>
   <si>
-    <t>cfg.6</t>
+    <t>cfg.4</t>
   </si>
   <si>
     <t xml:space="preserve">Do the same for loads and stores and AMOs where pmpcfg.X!=pmpcfg.W and X!=R to make sure that the X bit only affects instruction fetches.
 </t>
   </si>
   <si>
-    <t>cfg.7</t>
+    <t>cfg.5</t>
   </si>
   <si>
     <t>Perform instruction fetches of 32b instructions that straddle a boundary where each half is accessible but the other half gets an access fault based on pmpcfg.X.</t>
   </si>
   <si>
-    <t>cfg.8</t>
+    <t>cfg.6</t>
   </si>
   <si>
     <t>W</t>
@@ -101,35 +101,35 @@
 </t>
   </si>
   <si>
-    <t>cfg.9</t>
+    <t>cfg.7</t>
   </si>
   <si>
     <t xml:space="preserve">Do the same for loads where pmpcfg.R=1 and pmpcfg.W=0 to make sure that the W bit only affects stores and AMOs.
 </t>
   </si>
   <si>
-    <t>cfg.10</t>
+    <t>cfg.8</t>
   </si>
   <si>
     <t xml:space="preserve">Also, perform stores of 16b or greater to a misaligned address that straddle a boundary where each half is accessible but the other half gets an access fault based on pmpcfg.W.
 </t>
   </si>
   <si>
-    <t>cfg.11</t>
+    <t>cfg.9</t>
   </si>
   <si>
     <t xml:space="preserve">Foreach mode, foreach store and AMO instruction, perform the instruction referencing an address where the associated pmpcfg.W=0/1 and observe an access fault or not.
 </t>
   </si>
   <si>
-    <t>cfg.12</t>
+    <t>cfg.10</t>
   </si>
   <si>
     <t xml:space="preserve">Do the same for instruction fetches and loads where pmpcfg.W!=pmpcfg.X and R!=W (pruning illegal cases) to make sure that the W bit only affects stores and AMOs.
 </t>
   </si>
   <si>
-    <t>cfg.13</t>
+    <t>cfg.11</t>
   </si>
   <si>
     <t xml:space="preserve">Also, perform stores of 16b or greater to a misaligned address that straddle a boundary where each half is accessible but the other half gets an access fault based on pmpcfg.W.
@@ -137,7 +137,7 @@
 </t>
   </si>
   <si>
-    <t>cfg.14</t>
+    <t>cfg.12</t>
   </si>
   <si>
     <t>R</t>
@@ -147,35 +147,35 @@
 </t>
   </si>
   <si>
-    <t>cfg.15</t>
+    <t>cfg.13</t>
   </si>
   <si>
     <t xml:space="preserve">Do the same for stores where pmpcfg.R=1 and pmpcfg.W=0 to make sure that the R bit only affects loads and AMOs.
 </t>
   </si>
   <si>
-    <t>cfg.16</t>
+    <t>cfg.14</t>
   </si>
   <si>
     <t xml:space="preserve">Also, perform loads of 16b or greater to a misaligned address that straddle a boundary where each half is accessible but the other half gets an access fault based on pmpcfg.R.
 </t>
   </si>
   <si>
-    <t>cfg.17</t>
+    <t>cfg.15</t>
   </si>
   <si>
     <t xml:space="preserve">Foreach mode, foreach load and AMO instruction, perform the instruction referencing an address where the associated pmpcfg.R=0/1 and observe an access fault or not.
 </t>
   </si>
   <si>
-    <t>cfg.18</t>
+    <t>cfg.16</t>
   </si>
   <si>
     <t xml:space="preserve">Do the same for instruction fetches and stores where pmpcfg.R!=pmpcfg.X and R!=W (pruning illegal cases) to make sure that the R bit only affects loads and AMOs.
 </t>
   </si>
   <si>
-    <t>cfg.19</t>
+    <t>cfg.17</t>
   </si>
   <si>
     <t xml:space="preserve">Also, perform loads of 16b or greater to a misaligned address that straddle a boundary where each half is accessible but the other half gets an access fault based on pmpcfg.R.
@@ -183,21 +183,21 @@
 </t>
   </si>
   <si>
-    <t>cfg.20</t>
+    <t>cfg.18</t>
   </si>
   <si>
     <t xml:space="preserve">Foreach mode that is subject to table walks, foreach stage and level of table walks, perform memory accesses (load/store/AMO/inst fetch) that access a PTE at that stage/level where the associated pmpcfg.R=0/1 and observe an access fault or not.
 </t>
   </si>
   <si>
-    <t>cfg.21</t>
+    <t>cfg.19</t>
   </si>
   <si>
     <t xml:space="preserve">Foreach mode that is subject to table walks during 2-Stage Translation, foreach stage and level of table walks, perform memory accesses (load/store/AMO/inst fetch) that access a PTE at that stage/level where the associated pmpcfg.R=0/1 and observe an access fault or not.
 </t>
   </si>
   <si>
-    <t>cfg.22</t>
+    <t>cfg.20</t>
   </si>
   <si>
     <t>A</t>
@@ -207,7 +207,7 @@
 </t>
   </si>
   <si>
-    <t>addr.3</t>
+    <t>addr.1</t>
   </si>
   <si>
     <t>pmp addr</t>
@@ -244,7 +244,7 @@
 </t>
   </si>
   <si>
-    <t>cfg.23</t>
+    <t>cfg.21</t>
   </si>
   <si>
     <t>pmpcfg</t>
@@ -257,7 +257,7 @@
 </t>
   </si>
   <si>
-    <t>addr.4</t>
+    <t>addr.2</t>
   </si>
   <si>
     <t>pmpaddr</t>
@@ -270,7 +270,7 @@
 </t>
   </si>
   <si>
-    <t>cfg.24</t>
+    <t>cfg.22</t>
   </si>
   <si>
     <t>Locked bit</t>
@@ -280,7 +280,7 @@
 </t>
   </si>
   <si>
-    <t>cfg.25</t>
+    <t>cfg.23</t>
   </si>
   <si>
     <t>address range</t>
@@ -290,7 +290,7 @@
 </t>
   </si>
   <si>
-    <t>cfg.26</t>
+    <t>cfg.24</t>
   </si>
   <si>
     <t>special case1</t>
@@ -300,7 +300,7 @@
 </t>
   </si>
   <si>
-    <t>cfg.27</t>
+    <t>cfg.25</t>
   </si>
   <si>
     <t>special case2</t>
@@ -586,6 +586,28 @@
     <t xml:space="preserve">Aligned ld/st that crosses PMP boundary (PMP region is of 4 byte, and load double is crossing the boundary)
 </t>
   </si>
+  <si>
+    <t>addr.3</t>
+  </si>
+  <si>
+    <t>pmpaddr[063]</t>
+  </si>
+  <si>
+    <t>Writing to the CSR field
+(WARL)</t>
+  </si>
+  <si>
+    <t>Write waliking 1s and 0s to all pmpaddr CSRs in M mode</t>
+  </si>
+  <si>
+    <t>cfg.26</t>
+  </si>
+  <si>
+    <t>pmpcfg[015]</t>
+  </si>
+  <si>
+    <t>Write waliking 1s and 0s to all pmpcfg CSRs in M mode</t>
+  </si>
 </sst>
 </file>
 
@@ -628,7 +650,7 @@
     </font>
     <font/>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -651,6 +673,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE7F9EF"/>
         <bgColor rgb="FFE7F9EF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor theme="0"/>
       </patternFill>
     </fill>
   </fills>
@@ -704,7 +732,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -745,6 +773,18 @@
     <xf borderId="4" fillId="4" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="3" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="3" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -3207,14 +3247,28 @@
       <c r="X59" s="11"/>
     </row>
     <row r="60">
-      <c r="A60" s="4"/>
-      <c r="B60" s="4"/>
-      <c r="C60" s="4"/>
-      <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
-      <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
-      <c r="H60" s="4"/>
+      <c r="A60" s="16" t="s">
+        <v>170</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="C60" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="E60" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F60" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H60" s="10"/>
       <c r="I60" s="4"/>
       <c r="J60" s="4"/>
       <c r="K60" s="4"/>
@@ -3233,14 +3287,28 @@
       <c r="X60" s="4"/>
     </row>
     <row r="61">
-      <c r="A61" s="4"/>
-      <c r="B61" s="4"/>
-      <c r="C61" s="4"/>
-      <c r="D61" s="4"/>
-      <c r="E61" s="4"/>
-      <c r="F61" s="4"/>
-      <c r="G61" s="4"/>
-      <c r="H61" s="4"/>
+      <c r="A61" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="B61" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="C61" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="D61" s="18" t="s">
+        <v>176</v>
+      </c>
+      <c r="E61" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F61" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G61" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H61" s="10"/>
       <c r="I61" s="4"/>
       <c r="J61" s="4"/>
       <c r="K61" s="4"/>
@@ -25219,13 +25287,13 @@
     <mergeCell ref="B2:B21"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G2:G59">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G2:G61">
       <formula1>"Covered,Uncovered"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E59">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E61">
       <formula1>"Check against RM,Self Checking,Assertion Checker"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F59">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F61">
       <formula1>"To be Done,Done,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>